<commit_message>
update the separate workflows and lvl_studio independent of lvl_refraction
</commit_message>
<xml_diff>
--- a/projects/LVL_Erfurt/results/velocity/lvl_velocity_summary.xlsx
+++ b/projects/LVL_Erfurt/results/velocity/lvl_velocity_summary.xlsx
@@ -2,22 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="31590" yWindow="2175" windowWidth="23790" windowHeight="12735" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,15 +25,23 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00000000"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -43,7 +50,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002E4057"/>
+        <fgColor rgb="FF2E4057"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFD966"/>
       </patternFill>
     </fill>
     <fill>
@@ -64,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -72,9 +84,12 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -437,35 +452,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:AD4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
     <col width="5" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="10"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="13" max="14"/>
     <col width="9" customWidth="1" min="14" max="14"/>
     <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="16" max="17"/>
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="19" customWidth="1" min="18" max="18"/>
     <col width="16" customWidth="1" min="19" max="19"/>
     <col width="17" customWidth="1" min="20" max="20"/>
     <col width="18" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
-    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="23" max="24"/>
     <col width="11" customWidth="1" min="24" max="24"/>
     <col width="12" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="11" customWidth="1" min="26" max="27"/>
     <col width="11" customWidth="1" min="27" max="27"/>
     <col width="12" customWidth="1" min="28" max="28"/>
     <col width="11" customWidth="1" min="29" max="29"/>
@@ -518,42 +533,42 @@
           <t>V0C</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>V0</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>H0</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>TI1</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>H1</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>TI2</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>DR</t>
         </is>
@@ -630,7 +645,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LVLstudio</t>
+          <t>LVL150</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -641,69 +656,81 @@
           <t>192.5 m</t>
         </is>
       </c>
+      <c r="E2" t="n">
+        <v>639875.255</v>
+      </c>
+      <c r="F2" t="n">
+        <v>5655656.082</v>
+      </c>
+      <c r="G2" t="n">
+        <v>215.335</v>
+      </c>
       <c r="H2" t="n">
-        <v>344.826</v>
+        <v>457.209</v>
       </c>
       <c r="I2" t="n">
-        <v>376.304</v>
+        <v>450.313</v>
       </c>
       <c r="J2" t="n">
-        <v>348.459</v>
+        <v>475.571</v>
       </c>
       <c r="K2" t="n">
-        <v>7.607</v>
+        <v>5.576</v>
       </c>
       <c r="L2" t="n">
-        <v>1481.1</v>
+        <v>1947.753</v>
       </c>
       <c r="M2" t="n">
-        <v>42.435</v>
+        <v>22.742</v>
       </c>
       <c r="N2" t="n">
-        <v>29.882</v>
+        <v>20.572</v>
       </c>
       <c r="O2" t="n">
-        <v>3870.51</v>
+        <v>3241.633</v>
       </c>
       <c r="P2" t="n">
-        <v>80.764</v>
+        <v>40.084</v>
       </c>
       <c r="Q2" t="n">
-        <v>37.489</v>
+        <v>26.149</v>
       </c>
       <c r="R2" t="n">
         <v>192.5</v>
       </c>
       <c r="S2" t="n">
-        <v>192.5</v>
+        <v>196.791</v>
+      </c>
+      <c r="T2" t="n">
+        <v>24.51</v>
       </c>
       <c r="V2" t="n">
-        <v>397.072</v>
+        <v>385.373</v>
       </c>
       <c r="W2" t="n">
-        <v>292.58</v>
+        <v>529.046</v>
       </c>
       <c r="X2" t="n">
-        <v>1503.938</v>
+        <v>1884.046</v>
       </c>
       <c r="Y2" t="n">
-        <v>1415.884</v>
+        <v>2014.33</v>
       </c>
       <c r="Z2" t="n">
-        <v>1467.977</v>
+        <v>1945.281</v>
       </c>
       <c r="AA2" t="n">
-        <v>3889.703</v>
+        <v>3336.157</v>
       </c>
       <c r="AB2" t="n">
-        <v>0</v>
+        <v>3176.067</v>
       </c>
       <c r="AC2" t="n">
-        <v>3851.318</v>
+        <v>3278.24</v>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>2026-07-21 11:00:15</t>
+          <t>2026-07-23 14:10:28</t>
         </is>
       </c>
     </row>
@@ -713,7 +740,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LVLstudio_new</t>
+          <t>LVL155</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -721,77 +748,180 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>94.0 m</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>643407.669</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5652129.765</v>
+      </c>
+      <c r="G3" t="n">
+        <v>231.889</v>
+      </c>
+      <c r="H3" t="n">
+        <v>648.915</v>
+      </c>
+      <c r="I3" t="n">
+        <v>362.595</v>
+      </c>
+      <c r="J3" t="n">
+        <v>537.629</v>
+      </c>
+      <c r="K3" t="n">
+        <v>7.01</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2109.537</v>
+      </c>
+      <c r="M3" t="n">
+        <v>25.216</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>7.01</v>
+      </c>
+      <c r="R3" t="n">
+        <v>94</v>
+      </c>
+      <c r="S3" t="n">
+        <v>97.937</v>
+      </c>
+      <c r="T3" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="V3" t="n">
+        <v>622.379</v>
+      </c>
+      <c r="W3" t="n">
+        <v>675.451</v>
+      </c>
+      <c r="X3" t="n">
+        <v>2046.541</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>2126.088</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>1984.28</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>2026-07-23 14:21:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LVL721</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>192.5 m</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
-        <v>556.587</v>
-      </c>
-      <c r="I3" t="n">
-        <v>533.492</v>
-      </c>
-      <c r="J3" t="n">
-        <v>556.716</v>
-      </c>
-      <c r="K3" t="n">
-        <v>6.337</v>
-      </c>
-      <c r="L3" t="n">
-        <v>1842.443</v>
-      </c>
-      <c r="M3" t="n">
-        <v>21.7</v>
-      </c>
-      <c r="N3" t="n">
-        <v>20.509</v>
-      </c>
-      <c r="O3" t="n">
-        <v>3183.514</v>
-      </c>
-      <c r="P3" t="n">
-        <v>40.568</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>26.845</v>
-      </c>
-      <c r="R3" t="n">
+      <c r="E4" t="n">
+        <v>638915.632</v>
+      </c>
+      <c r="F4" t="n">
+        <v>5661065.306</v>
+      </c>
+      <c r="G4" t="n">
+        <v>202.414</v>
+      </c>
+      <c r="H4" t="n">
+        <v>615.14</v>
+      </c>
+      <c r="I4" t="n">
+        <v>645.995</v>
+      </c>
+      <c r="J4" t="n">
+        <v>621.322</v>
+      </c>
+      <c r="K4" t="n">
+        <v>4.594</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2380.58</v>
+      </c>
+      <c r="M4" t="n">
+        <v>14.274</v>
+      </c>
+      <c r="N4" t="n">
+        <v>15.007</v>
+      </c>
+      <c r="O4" t="n">
+        <v>3275.813</v>
+      </c>
+      <c r="P4" t="n">
+        <v>23.179</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>19.601</v>
+      </c>
+      <c r="R4" t="n">
         <v>192.5</v>
       </c>
-      <c r="S3" t="n">
-        <v>192.5</v>
-      </c>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="n">
-        <v>500.44</v>
-      </c>
-      <c r="W3" t="n">
-        <v>612.734</v>
-      </c>
-      <c r="X3" t="n">
-        <v>1809.961</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>1846.819</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>1846.724</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>3447.966</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>3057.468</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>3273.678</v>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>2026-07-21 13:15:16</t>
+      <c r="S4" t="n">
+        <v>198.567</v>
+      </c>
+      <c r="T4" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="n">
+        <v>340.599</v>
+      </c>
+      <c r="W4" t="n">
+        <v>889.6799999999999</v>
+      </c>
+      <c r="X4" t="n">
+        <v>2405</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>2499.131</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>2166.481</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>3351.735</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>3199.891</v>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>2026-07-23 15:21:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
updated GUI and picker
</commit_message>
<xml_diff>
--- a/projects/LVL_Erfurt/results/velocity/lvl_velocity_summary.xlsx
+++ b/projects/LVL_Erfurt/results/velocity/lvl_velocity_summary.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:AD13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -475,7 +475,7 @@
     <col width="19" customWidth="1" min="18" max="18"/>
     <col width="16" customWidth="1" min="19" max="19"/>
     <col width="17" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="27" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="24"/>
     <col width="11" customWidth="1" min="24" max="24"/>
@@ -1369,7 +1369,6 @@
       <c r="T9" t="n">
         <v>24.5</v>
       </c>
-      <c r="U9" t="inlineStr"/>
       <c r="V9" t="n">
         <v>504.326</v>
       </c>
@@ -1397,6 +1396,406 @@
       <c r="AD9" t="inlineStr">
         <is>
           <t>2026-07-27 14:12:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LVL151</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>94.0 m</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>640564.806</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5654989.79</v>
+      </c>
+      <c r="G10" t="n">
+        <v>219.275</v>
+      </c>
+      <c r="H10" t="n">
+        <v>438.448</v>
+      </c>
+      <c r="I10" t="n">
+        <v>558.633</v>
+      </c>
+      <c r="J10" t="n">
+        <v>518.2089999999999</v>
+      </c>
+      <c r="K10" t="n">
+        <v>4.885</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1857.424</v>
+      </c>
+      <c r="M10" t="n">
+        <v>18.106</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>4.885</v>
+      </c>
+      <c r="R10" t="n">
+        <v>94</v>
+      </c>
+      <c r="S10" t="n">
+        <v>99.809</v>
+      </c>
+      <c r="T10" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>2026-03-23 15:36:59 CET</t>
+        </is>
+      </c>
+      <c r="V10" t="n">
+        <v>387.89</v>
+      </c>
+      <c r="W10" t="n">
+        <v>489.005</v>
+      </c>
+      <c r="X10" t="n">
+        <v>1973.224</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>1782.801</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>1939.834</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>2026-07-28 10:03:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>LVL161</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>192.5 m</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>647630.568</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5648098.99</v>
+      </c>
+      <c r="G11" t="n">
+        <v>291.115</v>
+      </c>
+      <c r="H11" t="n">
+        <v>301.371</v>
+      </c>
+      <c r="I11" t="n">
+        <v>237.03</v>
+      </c>
+      <c r="J11" t="n">
+        <v>274.128</v>
+      </c>
+      <c r="K11" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1088.923</v>
+      </c>
+      <c r="M11" t="n">
+        <v>29.447</v>
+      </c>
+      <c r="N11" t="n">
+        <v>11.664</v>
+      </c>
+      <c r="O11" t="n">
+        <v>2268.958</v>
+      </c>
+      <c r="P11" t="n">
+        <v>48.999</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>15.835</v>
+      </c>
+      <c r="R11" t="n">
+        <v>192.5</v>
+      </c>
+      <c r="S11" t="n">
+        <v>197.793</v>
+      </c>
+      <c r="T11" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>2026-03-23 15:36:59 CET</t>
+        </is>
+      </c>
+      <c r="V11" t="n">
+        <v>325.051</v>
+      </c>
+      <c r="W11" t="n">
+        <v>277.691</v>
+      </c>
+      <c r="X11" t="n">
+        <v>1262.772</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>835.2430000000001</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>774.461</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>2413.485</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>2059.53</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>2204.473</v>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>2026-07-28 11:42:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>LVL151_new</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>94.0 m</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>640564.806</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5654989.79</v>
+      </c>
+      <c r="G12" t="n">
+        <v>219.275</v>
+      </c>
+      <c r="H12" t="n">
+        <v>424.386</v>
+      </c>
+      <c r="I12" t="n">
+        <v>558.633</v>
+      </c>
+      <c r="J12" t="n">
+        <v>511.179</v>
+      </c>
+      <c r="K12" t="n">
+        <v>4.913</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1880.708</v>
+      </c>
+      <c r="M12" t="n">
+        <v>18.498</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>4.913</v>
+      </c>
+      <c r="R12" t="n">
+        <v>94</v>
+      </c>
+      <c r="S12" t="n">
+        <v>99.809</v>
+      </c>
+      <c r="T12" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>2026-04-14 14:25:30 CEST</t>
+        </is>
+      </c>
+      <c r="V12" t="n">
+        <v>359.766</v>
+      </c>
+      <c r="W12" t="n">
+        <v>489.005</v>
+      </c>
+      <c r="X12" t="n">
+        <v>2066.36</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>1782.801</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>1939.834</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>2026-07-28 13:41:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>LVL161_new</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>192.5 m</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>647630.568</v>
+      </c>
+      <c r="F13" t="n">
+        <v>5648098.99</v>
+      </c>
+      <c r="G13" t="n">
+        <v>291.115</v>
+      </c>
+      <c r="H13" t="n">
+        <v>491.193</v>
+      </c>
+      <c r="I13" t="n">
+        <v>276.896</v>
+      </c>
+      <c r="J13" t="n">
+        <v>379.006</v>
+      </c>
+      <c r="K13" t="n">
+        <v>8.818</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2104.573</v>
+      </c>
+      <c r="M13" t="n">
+        <v>45.769</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>8.818</v>
+      </c>
+      <c r="R13" t="n">
+        <v>192.5</v>
+      </c>
+      <c r="S13" t="n">
+        <v>197.793</v>
+      </c>
+      <c r="T13" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>2026-04-16 17:33:54 CEST</t>
+        </is>
+      </c>
+      <c r="V13" t="n">
+        <v>342.506</v>
+      </c>
+      <c r="W13" t="n">
+        <v>639.88</v>
+      </c>
+      <c r="X13" t="n">
+        <v>2232.977</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>1880.719</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>2204.473</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>2026-07-28 14:18:57</t>
         </is>
       </c>
     </row>

</xml_diff>